<commit_message>
fix: return issue csv
</commit_message>
<xml_diff>
--- a/scenarios.xlsx
+++ b/scenarios.xlsx
@@ -23,10 +23,7 @@
     <t>Alignment</t>
   </si>
   <si>
-    <t>You need to run a few errands downtown which you think 
-may take you an hour. You go to your manager’s office at 
-work with whom you get on well and ask him to cover for 
-you. What do you say to him?</t>
+    <t>You need to run a few errands downtown which you think may take you an hour. You go to your manager’s office at work with whom you get on well and ask him to cover for you. What do you say to him?</t>
   </si>
   <si>
     <t>high</t>
@@ -200,6 +197,12 @@
     </font>
     <font>
       <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -208,12 +211,6 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -277,32 +274,32 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -620,11 +617,11 @@
   <dimension ref="A1:B51"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="10" width="63.71928571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="10" width="122.43357142857143" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5" customFormat="1" s="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1000,7 +997,7 @@
         <v>3</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75" customFormat="1" s="1">
       <c r="A48" s="3" t="s">
         <v>51</v>
       </c>
@@ -1008,7 +1005,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75" customFormat="1" s="1">
       <c r="A49" s="3" t="s">
         <v>52</v>
       </c>
@@ -1016,7 +1013,7 @@
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75" customFormat="1" s="1">
       <c r="A50" s="3" t="s">
         <v>53</v>
       </c>

</xml_diff>